<commit_message>
WB cost/coverage data - template and country databooks en/es/fr
</commit_message>
<xml_diff>
--- a/inputs/en/demo_national_input.xlsx
+++ b/inputs/en/demo_national_input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr saveExternalLinkValues="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tharindu.wickram\Desktop\Modeling\Nutrition\inputs\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC1CCE0-BD15-4384-BA57-6C1FA2F68ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A48A9ABD-4E96-42BD-8CB3-B326AB059902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="961" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="961" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline year population inputs" sheetId="1" r:id="rId1"/>
@@ -167,7 +167,7 @@
     <definedName name="term_SGA">'Baseline year population inputs'!$C$47</definedName>
     <definedName name="U5_mortality">'Baseline year population inputs'!$C$39</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcOnSave="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -13424,7 +13424,7 @@
         <v>171</v>
       </c>
       <c r="D5" s="102">
-        <v>1.73</v>
+        <v>2.17</v>
       </c>
       <c r="E5" s="102">
         <v>1</v>
@@ -13445,7 +13445,7 @@
         <v>170</v>
       </c>
       <c r="D6" s="102">
-        <v>1.73</v>
+        <v>2.17</v>
       </c>
       <c r="E6" s="102">
         <v>1</v>
@@ -13492,7 +13492,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="102">
-        <v>1.73</v>
+        <v>2.48</v>
       </c>
       <c r="F8" s="102">
         <v>1</v>
@@ -13513,7 +13513,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="102">
-        <v>1.73</v>
+        <v>2.48</v>
       </c>
       <c r="F9" s="102">
         <v>1</v>
@@ -13560,7 +13560,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="102">
-        <v>1.73</v>
+        <v>1.82</v>
       </c>
       <c r="G11" s="102">
         <v>1</v>
@@ -13581,7 +13581,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="102">
-        <v>1.73</v>
+        <v>1.82</v>
       </c>
       <c r="G12" s="102">
         <v>1</v>
@@ -13628,7 +13628,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="102">
-        <v>1.73</v>
+        <v>1.82</v>
       </c>
       <c r="H14" s="102">
         <v>1</v>
@@ -13649,7 +13649,7 @@
         <v>1</v>
       </c>
       <c r="G15" s="102">
-        <v>1.73</v>
+        <v>1.82</v>
       </c>
       <c r="H15" s="102">
         <v>1</v>
@@ -14490,7 +14490,7 @@
         <v>170</v>
       </c>
       <c r="D56" s="102">
-        <f t="shared" ref="D56:H59" si="1">IF(D3=1,1,D3*0.9)</f>
+        <f t="shared" ref="D56:H68" si="1">IF(D3=1,1,D3*0.9)</f>
         <v>1</v>
       </c>
       <c r="E56" s="102">
@@ -14544,7 +14544,7 @@
         <v>171</v>
       </c>
       <c r="D58" s="102">
-        <v>1.35</v>
+        <v>1.84</v>
       </c>
       <c r="E58" s="102">
         <f t="shared" si="1"/>
@@ -14569,7 +14569,7 @@
         <v>170</v>
       </c>
       <c r="D59" s="102">
-        <v>1.35</v>
+        <v>1.84</v>
       </c>
       <c r="E59" s="102">
         <f t="shared" si="1"/>
@@ -14610,7 +14610,7 @@
         <v>1</v>
       </c>
       <c r="H60" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -14626,7 +14626,7 @@
         <v>1</v>
       </c>
       <c r="E61" s="102">
-        <v>1.35</v>
+        <v>1.99</v>
       </c>
       <c r="F61" s="102">
         <f t="shared" si="2"/>
@@ -14637,7 +14637,7 @@
         <v>1</v>
       </c>
       <c r="H61" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
         <v>1</v>
       </c>
       <c r="E62" s="102">
-        <v>1.35</v>
+        <v>1.99</v>
       </c>
       <c r="F62" s="102">
         <f t="shared" si="2"/>
@@ -14662,7 +14662,7 @@
         <v>1</v>
       </c>
       <c r="H62" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -14688,7 +14688,7 @@
         <v>1</v>
       </c>
       <c r="H63" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -14708,14 +14708,14 @@
         <v>1</v>
       </c>
       <c r="F64" s="102">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="G64" s="102">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H64" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -14733,14 +14733,14 @@
         <v>1</v>
       </c>
       <c r="F65" s="102">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="G65" s="102">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H65" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -14766,7 +14766,7 @@
         <v>1</v>
       </c>
       <c r="H66" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -14790,10 +14790,10 @@
         <v>1</v>
       </c>
       <c r="G67" s="102">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="H67" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -14815,10 +14815,10 @@
         <v>1</v>
       </c>
       <c r="G68" s="102">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="H68" s="102">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -15827,7 +15827,7 @@
         <v>170</v>
       </c>
       <c r="D109" s="102">
-        <f t="shared" ref="D109:H112" si="8">IF(D3=1,1,D3*1.05)</f>
+        <f t="shared" ref="D109:H121" si="8">IF(D3=1,1,D3*1.05)</f>
         <v>1</v>
       </c>
       <c r="E109" s="102">
@@ -15881,18 +15881,18 @@
         <v>171</v>
       </c>
       <c r="D111" s="102">
-        <v>2.11</v>
+        <v>2.56</v>
       </c>
       <c r="E111" s="102">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="E111:G112" si="9">IF(E58=1,1,E58*0.9)</f>
         <v>1</v>
       </c>
       <c r="F111" s="102">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="G111" s="102">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="H111" s="102">
@@ -15906,18 +15906,18 @@
         <v>170</v>
       </c>
       <c r="D112" s="102">
-        <v>2.11</v>
+        <v>2.56</v>
       </c>
       <c r="E112" s="102">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="F112" s="102">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="G112" s="102">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="H112" s="102">
@@ -15931,23 +15931,23 @@
         <v>169</v>
       </c>
       <c r="D113" s="102">
-        <f t="shared" ref="D113:H123" si="9">IF(D7=1,1,D7*1.05)</f>
+        <f t="shared" ref="D113:G121" si="10">IF(D60=1,1,D60*0.9)</f>
         <v>1</v>
       </c>
       <c r="E113" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="F113" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="G113" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="H113" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -15959,22 +15959,22 @@
         <v>171</v>
       </c>
       <c r="D114" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E114" s="102">
-        <v>2.11</v>
+        <v>3.09</v>
       </c>
       <c r="F114" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="G114" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="H114" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -15984,22 +15984,22 @@
         <v>170</v>
       </c>
       <c r="D115" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E115" s="102">
-        <v>2.11</v>
+        <v>3.09</v>
       </c>
       <c r="F115" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="G115" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="H115" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -16009,23 +16009,23 @@
         <v>169</v>
       </c>
       <c r="D116" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E116" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="F116" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="G116" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="H116" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -16037,22 +16037,22 @@
         <v>171</v>
       </c>
       <c r="D117" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E117" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="F117" s="102">
-        <v>2.11</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="G117" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="H117" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -16062,22 +16062,22 @@
         <v>170</v>
       </c>
       <c r="D118" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E118" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="F118" s="102">
-        <v>2.11</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="G118" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="H118" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -16087,23 +16087,23 @@
         <v>169</v>
       </c>
       <c r="D119" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E119" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="F119" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="G119" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="H119" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -16115,22 +16115,22 @@
         <v>171</v>
       </c>
       <c r="D120" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E120" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="F120" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="G120" s="102">
-        <v>2.11</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="H120" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -16140,22 +16140,22 @@
         <v>170</v>
       </c>
       <c r="D121" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E121" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="F121" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="G121" s="102">
-        <v>2.11</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="H121" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -16165,23 +16165,23 @@
         <v>169</v>
       </c>
       <c r="D122" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="D122:H123" si="11">IF(D16=1,1,D16*1.05)</f>
         <v>1</v>
       </c>
       <c r="E122" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="F122" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="G122" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="H122" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
     </row>
@@ -16193,23 +16193,23 @@
         <v>169</v>
       </c>
       <c r="D123" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1.1025</v>
       </c>
       <c r="E123" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1.1025</v>
       </c>
       <c r="F123" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1.1025</v>
       </c>
       <c r="G123" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1.1025</v>
       </c>
       <c r="H123" s="102">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
     </row>
@@ -16235,19 +16235,19 @@
         <v>1</v>
       </c>
       <c r="E125" s="102">
-        <f t="shared" ref="E125:H125" si="10">IF(E19=1,1,E19*1.05)</f>
+        <f t="shared" ref="E125:H125" si="12">IF(E19=1,1,E19*1.05)</f>
         <v>1</v>
       </c>
       <c r="F125" s="102">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G125" s="102">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H125" s="102">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
     </row>
@@ -16257,23 +16257,23 @@
         <v>170</v>
       </c>
       <c r="D126" s="102">
-        <f t="shared" ref="D126:H140" si="11">IF(D20=1,1,D20*1.05)</f>
+        <f t="shared" ref="D126:H140" si="13">IF(D20=1,1,D20*1.05)</f>
         <v>1</v>
       </c>
       <c r="E126" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F126" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G126" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H126" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16283,23 +16283,23 @@
         <v>169</v>
       </c>
       <c r="D127" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E127" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F127" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G127" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H127" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16311,23 +16311,23 @@
         <v>171</v>
       </c>
       <c r="D128" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E128" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F128" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G128" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H128" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16337,23 +16337,23 @@
         <v>170</v>
       </c>
       <c r="D129" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E129" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F129" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G129" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H129" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16363,23 +16363,23 @@
         <v>169</v>
       </c>
       <c r="D130" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E130" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F130" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G130" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H130" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16391,23 +16391,23 @@
         <v>171</v>
       </c>
       <c r="D131" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E131" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F131" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G131" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H131" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16417,23 +16417,23 @@
         <v>170</v>
       </c>
       <c r="D132" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E132" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F132" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G132" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H132" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16443,23 +16443,23 @@
         <v>169</v>
       </c>
       <c r="D133" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E133" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F133" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G133" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H133" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16471,23 +16471,23 @@
         <v>171</v>
       </c>
       <c r="D134" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E134" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F134" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G134" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H134" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16497,23 +16497,23 @@
         <v>170</v>
       </c>
       <c r="D135" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E135" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F135" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G135" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H135" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16523,23 +16523,23 @@
         <v>169</v>
       </c>
       <c r="D136" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E136" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F136" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G136" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H136" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16551,23 +16551,23 @@
         <v>171</v>
       </c>
       <c r="D137" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E137" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F137" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G137" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H137" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16577,23 +16577,23 @@
         <v>170</v>
       </c>
       <c r="D138" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E138" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F138" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G138" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H138" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16603,23 +16603,23 @@
         <v>169</v>
       </c>
       <c r="D139" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E139" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F139" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G139" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H139" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16631,23 +16631,23 @@
         <v>169</v>
       </c>
       <c r="D140" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E140" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F140" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G140" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H140" s="102">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -16673,19 +16673,19 @@
         <v>1</v>
       </c>
       <c r="E142" s="102">
-        <f t="shared" ref="E142:H142" si="12">IF(E36=1,1,E36*1.05)</f>
+        <f t="shared" ref="E142:H142" si="14">IF(E36=1,1,E36*1.05)</f>
         <v>1</v>
       </c>
       <c r="F142" s="102">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="G142" s="102">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="H142" s="102">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
     </row>
@@ -16695,23 +16695,23 @@
         <v>170</v>
       </c>
       <c r="D143" s="102">
-        <f t="shared" ref="D143:H157" si="13">IF(D37=1,1,D37*1.05)</f>
+        <f t="shared" ref="D143:H157" si="15">IF(D37=1,1,D37*1.05)</f>
         <v>1</v>
       </c>
       <c r="E143" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F143" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G143" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H143" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16721,23 +16721,23 @@
         <v>169</v>
       </c>
       <c r="D144" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E144" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F144" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G144" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H144" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16749,23 +16749,23 @@
         <v>171</v>
       </c>
       <c r="D145" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E145" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F145" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G145" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H145" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16775,23 +16775,23 @@
         <v>170</v>
       </c>
       <c r="D146" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E146" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F146" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G146" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H146" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16801,23 +16801,23 @@
         <v>169</v>
       </c>
       <c r="D147" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E147" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F147" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G147" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H147" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16829,23 +16829,23 @@
         <v>171</v>
       </c>
       <c r="D148" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E148" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F148" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G148" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H148" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16855,23 +16855,23 @@
         <v>170</v>
       </c>
       <c r="D149" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E149" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F149" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G149" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H149" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16881,23 +16881,23 @@
         <v>169</v>
       </c>
       <c r="D150" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E150" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F150" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G150" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H150" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16909,23 +16909,23 @@
         <v>171</v>
       </c>
       <c r="D151" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E151" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F151" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G151" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H151" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16935,23 +16935,23 @@
         <v>170</v>
       </c>
       <c r="D152" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E152" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F152" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G152" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H152" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16961,23 +16961,23 @@
         <v>169</v>
       </c>
       <c r="D153" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E153" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F153" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G153" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H153" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -16989,23 +16989,23 @@
         <v>171</v>
       </c>
       <c r="D154" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E154" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F154" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G154" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H154" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -17015,23 +17015,23 @@
         <v>170</v>
       </c>
       <c r="D155" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E155" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F155" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G155" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H155" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -17041,23 +17041,23 @@
         <v>169</v>
       </c>
       <c r="D156" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E156" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F156" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G156" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H156" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
@@ -17069,35 +17069,59 @@
         <v>169</v>
       </c>
       <c r="D157" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E157" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="F157" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="G157" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="H157" s="102">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="PJvvczTX02udclIHc4BYVrFcnDWQgrEMznGaMDqc9c7dODneUitm4zod0zPOcMmikisDTo5XoDZbroNh1SOQlQ==" saltValue="d6DJlx6zmP+EipmKY6bfHA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="3MNi0HHfsvbKBTuSA5lQSLhlW//BMbBefosk4swt5SLv2tmpBbkcGSlWseFBRMQQOk+e3uORbQ5FcRsh4E4JvA==" saltValue="9yz037DEjTrccL9vy4gweA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="45">
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="B148:B150"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="B134:B136"/>
+    <mergeCell ref="B137:B139"/>
+    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B116"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B89:B91"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="B98:B100"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B67:B69"/>
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="B45:B47"/>
     <mergeCell ref="B48:B50"/>
@@ -17107,36 +17131,12 @@
     <mergeCell ref="B31:B33"/>
     <mergeCell ref="B36:B38"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B89:B91"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="B98:B100"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B116"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="B148:B150"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="B134:B136"/>
-    <mergeCell ref="B137:B139"/>
-    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -26484,7 +26484,7 @@
       <c r="I328" s="92"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="z5qzIi1ZlGssU/OiYY7WWiJoR1TaHnOOh+cFwOn3BpdV8g3fDSuCKM2FT4tYtp77DPGMVtU7PzAWhrFcFrpEMg==" saltValue="qsszEe2oCJFCGTnlInMljg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="MBta6JwcN4aprXgE/6TMmpGZPA4pG7IVPUgKb9CMlkSlLUZb++bcBUuHPKxJylRrVSnAyg+0kX1qjB7uB3jCdQ==" saltValue="bhFmTLnxXPc7o3gdjKF6Fg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <legacyDrawing r:id="rId1"/>
@@ -26680,7 +26680,7 @@
         <v>190</v>
       </c>
       <c r="C12" s="104">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D12" s="104">
         <v>1.39</v>
@@ -27016,7 +27016,7 @@
         <v>282</v>
       </c>
       <c r="C35" s="104">
-        <v>1.26</v>
+        <v>1</v>
       </c>
       <c r="D35" s="104">
         <v>1.1100000000000001</v>
@@ -27372,7 +27372,7 @@
         <v>292</v>
       </c>
       <c r="C58" s="104">
-        <v>1.78</v>
+        <v>1</v>
       </c>
       <c r="D58" s="104">
         <v>1.74</v>
@@ -27521,12 +27521,9 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="2aTOkQvcsuJWBOLN2ckjI7KHl3V854l5vTCVkfcr0ANH8QApmmuHtG/XADuSye+bDx7h4bFWV7MSCTfUmZWoCw==" saltValue="0Mt/Wzxt/AYjzZ0BBVBN/Q==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="QAVwj9PWadQcYcL52alW/JJQquT7j6uGPCclqgaz9+O8krRpbbsh1HExJbjXqiYNshQdlMMFo0ZnrWFakvrKaA==" saltValue="caoeAy2KJFZFYGAg6OWiLw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
-  <ignoredErrors>
-    <ignoredError sqref="C29:G32 D26:G26 C39:G40 C52:G54 C55:G55 D49:G49 C63:G63" unlockedFormula="1"/>
-  </ignoredErrors>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -28345,7 +28342,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="y0vFCUr6jQyY6zQBRlULLcVrg53Rq8yOs7wqPgO6lP26Nps2Fs/G1qUtWXIJ+6MZpSkLaCYJ5rBXvS6Vsp0C5w==" saltValue="ZZUBAtW4ABLI8WN+D6FzKQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="VNqV9laeHLEmOvMS2HGD5bmuz3IT62zAHDRQ56J67ZOBCPkqTbLk45H+TOI55sQOIALXqxS0CNWqR8cFOBHQ/Q==" saltValue="hKf7DQYsC+E7vW3zy5NTxQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
 </worksheet>
@@ -28421,10 +28418,10 @@
         <v>0.92</v>
       </c>
       <c r="D3" s="104">
-        <v>0.53</v>
+        <v>0.92</v>
       </c>
       <c r="E3" s="104">
-        <v>1</v>
+        <v>0.92</v>
       </c>
       <c r="F3" s="104">
         <v>1</v>
@@ -29232,14 +29229,13 @@
         <v>0.87</v>
       </c>
       <c r="D26" s="104">
-        <v>0.4</v>
+        <v>0.87</v>
       </c>
       <c r="E26" s="104">
-        <f t="shared" ref="E26:O26" si="1">IF(E3=1,1,E3*0.9)</f>
-        <v>1</v>
+        <v>0.87</v>
       </c>
       <c r="F26" s="104">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="F26:O26" si="1">IF(F3=1,1,F3*0.9)</f>
         <v>1</v>
       </c>
       <c r="G26" s="104">
@@ -30161,14 +30157,13 @@
         <v>0.99</v>
       </c>
       <c r="D49" s="104">
-        <v>0.7</v>
+        <v>0.99</v>
       </c>
       <c r="E49" s="104">
-        <f t="shared" ref="E49:O49" si="5">IF(E3=1,1,E3*1.05)</f>
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="F49" s="104">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="F49:O49" si="5">IF(F3=1,1,F3*1.05)</f>
         <v>1</v>
       </c>
       <c r="G49" s="104">
@@ -31031,7 +31026,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="NCGswl3bk6pRR//Ip+G0p1q0x8CSdirliKLz4dR3alBBXFKnAUJP7W9cZlp4Q9a5Zihxr509AhcGp3Drkh9nzQ==" saltValue="x95/MdDL5rJcAyM6I7v1QQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="1H36YeFo+tYWK8ppDEqRt9VLAlN4fhiSrdsiceTY84S0a72cFwg9qXz4yszhjj9aJElQkYzzqKoVekKKS4PDuQ==" saltValue="rTLJ2c1Dod8ZlB3HOpXo6A==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
 </worksheet>
@@ -31959,19 +31954,19 @@
         <v>262</v>
       </c>
       <c r="D28" s="104">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E28" s="104">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="F28" s="104">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="G28" s="104">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="H28" s="104">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -33213,19 +33208,19 @@
         <v>262</v>
       </c>
       <c r="D83" s="104">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E83" s="104">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F83" s="104">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G83" s="104">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H83" s="104">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -34472,19 +34467,19 @@
         <v>262</v>
       </c>
       <c r="D138" s="104">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="E138" s="104">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="F138" s="104">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="G138" s="104">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="H138" s="104">
-        <v>0</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.25">
@@ -35049,7 +35044,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="pJuCxRkuJTNVQMXzzuWGNE8Rrsg3d47K9SpmDEM5DcFgC2uns7HIEVwwfl/+461WSpTiJHa0KUHO5B858n+jvA==" saltValue="iEtCZOa8GN8kcnGn6gdz8Q==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="X00FxclSNSjJirmMy+z7qEOva6bgZMAswwg9/Zx2Czg7XdgCu39+BpOdZzILyc/8IAiCsVCp13t6IIjdq7Xvvg==" saltValue="yzgPEUxGLJUP683C8Cv0IA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
 </worksheet>

</xml_diff>

<commit_message>
databook update for stillbirth
</commit_message>
<xml_diff>
--- a/inputs/en/demo_national_input.xlsx
+++ b/inputs/en/demo_national_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tharindu.wickram\Desktop\Modeling\2025 studies\Nutrition\inputs\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4DB93BC-E507-44CA-A384-3E73B9F83914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0037AD-FCE1-4434-AC08-DDCD99D961FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="904" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="904" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline year population inputs" sheetId="1" r:id="rId1"/>
@@ -244,7 +244,8 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Placeholders currently</t>
+RR = 0.91 (0.86-0.98)
+Hofmeyr et al 2023 </t>
         </r>
       </text>
     </comment>
@@ -17638,12 +17639,36 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="3MNi0HHfsvbKBTuSA5lQSLhlW//BMbBefosk4swt5SLv2tmpBbkcGSlWseFBRMQQOk+e3uORbQ5FcRsh4E4JvA==" saltValue="9yz037DEjTrccL9vy4gweA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="45">
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="B148:B150"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="B134:B136"/>
+    <mergeCell ref="B137:B139"/>
+    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B116"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B89:B91"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="B98:B100"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B67:B69"/>
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="B45:B47"/>
     <mergeCell ref="B48:B50"/>
@@ -17653,36 +17678,12 @@
     <mergeCell ref="B31:B33"/>
     <mergeCell ref="B36:B38"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B89:B91"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="B98:B100"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B116"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="B148:B150"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="B134:B136"/>
-    <mergeCell ref="B137:B139"/>
-    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -35973,16 +35974,16 @@
         <v>157</v>
       </c>
       <c r="D9" s="104">
-        <v>0.59</v>
+        <v>0.09</v>
       </c>
       <c r="E9" s="104">
-        <v>0.59</v>
+        <v>0.09</v>
       </c>
       <c r="F9" s="104">
-        <v>0.59</v>
+        <v>0.09</v>
       </c>
       <c r="G9" s="104">
-        <v>0.59</v>
+        <v>0.09</v>
       </c>
       <c r="H9" s="31"/>
     </row>
@@ -36184,20 +36185,16 @@
         <v>157</v>
       </c>
       <c r="D20" s="104">
-        <f t="shared" ref="D20:G20" si="3">IF($C9="Affected fraction",D9,IF(D9=1,1,D9*0.9))</f>
-        <v>0.53100000000000003</v>
+        <v>0.02</v>
       </c>
       <c r="E20" s="104">
-        <f t="shared" si="3"/>
-        <v>0.53100000000000003</v>
+        <v>0.02</v>
       </c>
       <c r="F20" s="104">
-        <f t="shared" si="3"/>
-        <v>0.53100000000000003</v>
+        <v>0.02</v>
       </c>
       <c r="G20" s="104">
-        <f t="shared" si="3"/>
-        <v>0.53100000000000003</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="22" spans="1:7" s="106" customFormat="1" ht="13" x14ac:dyDescent="0.3">
@@ -36241,15 +36238,15 @@
         <v>1</v>
       </c>
       <c r="E24" s="104">
-        <f t="shared" ref="E24:G24" si="4">IF($C2="Affected fraction",E2,IF(E2=1,1,E2*1.05))</f>
+        <f t="shared" ref="E24:G24" si="3">IF($C2="Affected fraction",E2,IF(E2=1,1,E2*1.05))</f>
         <v>1</v>
       </c>
       <c r="F24" s="104">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G24" s="104">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
@@ -36281,19 +36278,19 @@
         <v>261</v>
       </c>
       <c r="D26" s="104">
-        <f t="shared" ref="D26:G26" si="5">IF($C4="Affected fraction",D4,IF(D4=1,1,D4*1.05))</f>
+        <f t="shared" ref="D26:G26" si="4">IF($C4="Affected fraction",D4,IF(D4=1,1,D4*1.05))</f>
         <v>1</v>
       </c>
       <c r="E26" s="104">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="F26" s="104">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="G26" s="104">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
     </row>
@@ -36306,15 +36303,15 @@
         <v>0.64900000000000002</v>
       </c>
       <c r="E27" s="104">
-        <f t="shared" ref="E27:G27" si="6">IF($C5="Affected fraction",E5,IF(E5=1,1,E5*1.1))</f>
+        <f t="shared" ref="E27:G27" si="5">IF($C5="Affected fraction",E5,IF(E5=1,1,E5*1.1))</f>
         <v>0.64900000000000002</v>
       </c>
       <c r="F27" s="104">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>0.64900000000000002</v>
       </c>
       <c r="G27" s="104">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>0.64900000000000002</v>
       </c>
     </row>
@@ -36329,19 +36326,19 @@
         <v>261</v>
       </c>
       <c r="D28" s="104">
-        <f t="shared" ref="D28:G28" si="7">IF($C6="Affected fraction",D6,IF(D6=1,1,D6*1.05))</f>
+        <f t="shared" ref="D28:G28" si="6">IF($C6="Affected fraction",D6,IF(D6=1,1,D6*1.05))</f>
         <v>1</v>
       </c>
       <c r="E28" s="104">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="F28" s="104">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="G28" s="104">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -36354,15 +36351,15 @@
         <v>0.64900000000000002</v>
       </c>
       <c r="E29" s="104">
-        <f t="shared" ref="E29:G29" si="8">IF($C7="Affected fraction",E7,IF(E7=1,1,E7*1.1))</f>
+        <f t="shared" ref="E29:G29" si="7">IF($C7="Affected fraction",E7,IF(E7=1,1,E7*1.1))</f>
         <v>0.64900000000000002</v>
       </c>
       <c r="F29" s="104">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0.64900000000000002</v>
       </c>
       <c r="G29" s="104">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0.64900000000000002</v>
       </c>
     </row>
@@ -36377,19 +36374,19 @@
         <v>261</v>
       </c>
       <c r="D30" s="104">
-        <f t="shared" ref="D30:G30" si="9">IF($C8="Affected fraction",D8,IF(D8=1,1,D8*1.05))</f>
+        <f t="shared" ref="D30:G30" si="8">IF($C8="Affected fraction",D8,IF(D8=1,1,D8*1.05))</f>
         <v>1</v>
       </c>
       <c r="E30" s="104">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="F30" s="104">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="G30" s="104">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -36398,24 +36395,20 @@
         <v>157</v>
       </c>
       <c r="D31" s="104">
-        <f>IF($C9="Affected fraction",D9,IF(D9=1,1,D9*1.1))</f>
-        <v>0.64900000000000002</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E31" s="104">
-        <f t="shared" ref="E31:G31" si="10">IF($C9="Affected fraction",E9,IF(E9=1,1,E9*1.1))</f>
-        <v>0.64900000000000002</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="F31" s="104">
-        <f t="shared" si="10"/>
-        <v>0.64900000000000002</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="G31" s="104">
-        <f t="shared" si="10"/>
-        <v>0.64900000000000002</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="s9mtpHs5kU1m2pYBBKLgia/vjx39im+kzmvtlB7yk6tHJM6pmyokGGByPY/xREVz/tHwT1FKVdGnOC7360YG4w==" saltValue="1lIKzNfSgC+G2y+SfnzxOw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="9gpYHKgj6UpVVviN7uxazCUWSTWVQZxWndpvCAxXJ0y6bbqG2bj+A9gvoQzXvuQCJzoAAyx1qKZvUYataGoRuA==" saltValue="kap3hl33opxMDisBGx+upA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
cash transfer only for 6-23 months
</commit_message>
<xml_diff>
--- a/inputs/en/demo_national_input.xlsx
+++ b/inputs/en/demo_national_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tharindu.wickram\Desktop\Modeling\2025 studies\Nutrition\inputs\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0037AD-FCE1-4434-AC08-DDCD99D961FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFF41C8-5088-46B8-952F-0E3A1364B9B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="904" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="904" firstSheet="7" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline year population inputs" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <sheet name="Program dependencies" sheetId="58" r:id="rId11"/>
     <sheet name="Reference programs" sheetId="59" state="hidden" r:id="rId12"/>
     <sheet name="Incidence of conditions" sheetId="7" state="hidden" r:id="rId13"/>
-    <sheet name="Programs target population" sheetId="21" state="hidden" r:id="rId14"/>
+    <sheet name="Programs target population" sheetId="21" r:id="rId14"/>
     <sheet name="Cost curve options" sheetId="61" state="hidden" r:id="rId15"/>
     <sheet name="Programs family planning" sheetId="54" state="hidden" r:id="rId16"/>
     <sheet name="Programs impacted population" sheetId="62" state="hidden" r:id="rId17"/>
@@ -7838,8 +7838,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="69">
-        <f>food_insecure</f>
-        <v>0.28199999999999997</v>
+        <v>0</v>
       </c>
       <c r="E2" s="69">
         <f>food_insecure</f>
@@ -7850,8 +7849,7 @@
         <v>0.28199999999999997</v>
       </c>
       <c r="G2" s="69">
-        <f>food_insecure</f>
-        <v>0.28199999999999997</v>
+        <v>0</v>
       </c>
       <c r="H2" s="70">
         <v>0</v>
@@ -8460,16 +8458,20 @@
         <v>0</v>
       </c>
       <c r="H16" s="69">
-        <v>1</v>
+        <f>food_insecure</f>
+        <v>0.28199999999999997</v>
       </c>
       <c r="I16" s="69">
-        <v>1</v>
+        <f>food_insecure</f>
+        <v>0.28199999999999997</v>
       </c>
       <c r="J16" s="69">
-        <v>1</v>
+        <f>food_insecure</f>
+        <v>0.28199999999999997</v>
       </c>
       <c r="K16" s="69">
-        <v>1</v>
+        <f>food_insecure</f>
+        <v>0.28199999999999997</v>
       </c>
       <c r="L16" s="70">
         <v>0</v>
@@ -17639,6 +17641,42 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="3MNi0HHfsvbKBTuSA5lQSLhlW//BMbBefosk4swt5SLv2tmpBbkcGSlWseFBRMQQOk+e3uORbQ5FcRsh4E4JvA==" saltValue="9yz037DEjTrccL9vy4gweA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="45">
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B67:B69"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B89:B91"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="B98:B100"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B116"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="B125:B127"/>
     <mergeCell ref="B145:B147"/>
     <mergeCell ref="B148:B150"/>
     <mergeCell ref="B151:B153"/>
@@ -17648,42 +17686,6 @@
     <mergeCell ref="B134:B136"/>
     <mergeCell ref="B137:B139"/>
     <mergeCell ref="B142:B144"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B116"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B89:B91"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="B98:B100"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
wrappers for translations and optimization testing on stillbirths
</commit_message>
<xml_diff>
--- a/inputs/en/demo_national_input.xlsx
+++ b/inputs/en/demo_national_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tharindu.wickram\Desktop\Modeling\2025 studies\Nutrition\inputs\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFF41C8-5088-46B8-952F-0E3A1364B9B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176A65D2-E30F-4F50-A53B-83CAF0FAAB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="904" firstSheet="7" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="904" firstSheet="7" activeTab="27" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline year population inputs" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <sheet name="Programs anaemia" sheetId="70" state="hidden" r:id="rId25"/>
     <sheet name="Programs wasting" sheetId="71" state="hidden" r:id="rId26"/>
     <sheet name="Programs for children" sheetId="72" state="hidden" r:id="rId27"/>
-    <sheet name="Programs for PW" sheetId="73" state="hidden" r:id="rId28"/>
+    <sheet name="Programs for PW" sheetId="73" r:id="rId28"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId29"/>
@@ -8409,19 +8409,19 @@
         <v>0</v>
       </c>
       <c r="H15" s="69">
-        <f>food_insecure</f>
+        <f t="shared" ref="H15:K16" si="0">food_insecure</f>
         <v>0.28199999999999997</v>
       </c>
       <c r="I15" s="69">
-        <f>food_insecure</f>
+        <f t="shared" si="0"/>
         <v>0.28199999999999997</v>
       </c>
       <c r="J15" s="69">
-        <f>food_insecure</f>
+        <f t="shared" si="0"/>
         <v>0.28199999999999997</v>
       </c>
       <c r="K15" s="69">
-        <f>food_insecure</f>
+        <f t="shared" si="0"/>
         <v>0.28199999999999997</v>
       </c>
       <c r="L15" s="70">
@@ -8458,19 +8458,19 @@
         <v>0</v>
       </c>
       <c r="H16" s="69">
-        <f>food_insecure</f>
+        <f t="shared" si="0"/>
         <v>0.28199999999999997</v>
       </c>
       <c r="I16" s="69">
-        <f>food_insecure</f>
+        <f t="shared" si="0"/>
         <v>0.28199999999999997</v>
       </c>
       <c r="J16" s="69">
-        <f>food_insecure</f>
+        <f t="shared" si="0"/>
         <v>0.28199999999999997</v>
       </c>
       <c r="K16" s="69">
-        <f>food_insecure</f>
+        <f t="shared" si="0"/>
         <v>0.28199999999999997</v>
       </c>
       <c r="L16" s="70">
@@ -9035,47 +9035,47 @@
         <v>0</v>
       </c>
       <c r="E30" s="69">
-        <f t="shared" ref="E30:O30" si="0">frac_maize</f>
+        <f t="shared" ref="E30:O30" si="1">frac_maize</f>
         <v>0.8</v>
       </c>
       <c r="F30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="G30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="H30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="I30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="J30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="K30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="L30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="M30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="N30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
       <c r="O30" s="69">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
     </row>
@@ -9090,47 +9090,47 @@
         <v>0</v>
       </c>
       <c r="E31" s="69">
-        <f t="shared" ref="E31:O31" si="1">frac_rice</f>
+        <f t="shared" ref="E31:O31" si="2">frac_rice</f>
         <v>0.1</v>
       </c>
       <c r="F31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="G31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="H31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="I31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="J31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="K31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="L31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="M31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="N31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O31" s="69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
     </row>
@@ -9149,43 +9149,43 @@
         <v>0.1</v>
       </c>
       <c r="F32" s="69">
-        <f t="shared" ref="F32:O32" si="2">frac_wheat</f>
+        <f t="shared" ref="F32:O32" si="3">frac_wheat</f>
         <v>0.1</v>
       </c>
       <c r="G32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="H32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="I32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="J32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="K32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="L32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="M32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="N32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="O32" s="69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
     </row>
@@ -9238,55 +9238,55 @@
         <v>34</v>
       </c>
       <c r="C34" s="69">
-        <f t="shared" ref="C34:O34" si="3">frac_malaria_risk</f>
+        <f t="shared" ref="C34:O34" si="4">frac_malaria_risk</f>
         <v>1</v>
       </c>
       <c r="D34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="E34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="F34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="G34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="H34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="L34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="M34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="N34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="O34" s="69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
     </row>
@@ -17641,12 +17641,36 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="3MNi0HHfsvbKBTuSA5lQSLhlW//BMbBefosk4swt5SLv2tmpBbkcGSlWseFBRMQQOk+e3uORbQ5FcRsh4E4JvA==" saltValue="9yz037DEjTrccL9vy4gweA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="45">
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="B148:B150"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="B134:B136"/>
+    <mergeCell ref="B137:B139"/>
+    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B116"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B89:B91"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="B98:B100"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B67:B69"/>
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="B45:B47"/>
     <mergeCell ref="B48:B50"/>
@@ -17656,36 +17680,12 @@
     <mergeCell ref="B31:B33"/>
     <mergeCell ref="B36:B38"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B89:B91"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="B98:B100"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B116"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="B148:B150"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="B134:B136"/>
-    <mergeCell ref="B137:B139"/>
-    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>